<commit_message>
update config for liyang.tjtj@gmail.com
</commit_message>
<xml_diff>
--- a/configuration/name_list.xlsx
+++ b/configuration/name_list.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4880" yWindow="500" windowWidth="46320" windowHeight="26640" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="list" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="list" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -516,7 +516,11 @@
           <t>ceshizhanghao31900@outlook.com</t>
         </is>
       </c>
-      <c r="B2" s="0" t="n"/>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>fxmanofndzdpbtbm</t>
+        </is>
+      </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
           <t>PassWord~1915</t>
@@ -596,7 +600,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>liyang.tjtj@gmail.com</t>
+          <t>dummy@dummy.com</t>
         </is>
       </c>
     </row>
@@ -615,17 +619,21 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ceshizhanghao31901@outlook.com</t>
-        </is>
-      </c>
-      <c r="B7" s="0" t="n"/>
+          <t>ceshizhanghao31901@gmail.com</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>gmunjnrjqwxbugrk</t>
+        </is>
+      </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>PassWord~9817</t>
+          <t>PassWord~c4d</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>45658.98274305555</v>
+        <v>45689.98274305555</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
@@ -638,10 +646,14 @@
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>5746 位置1</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n"/>
+          <t>1311 位置1</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>liyang.tjtj@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="G8" s="2" t="n"/>
@@ -769,9 +781,10 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" verticalDpi="0"/>

</xml_diff>

<commit_message>
remove liyang from name list
</commit_message>
<xml_diff>
--- a/configuration/name_list.xlsx
+++ b/configuration/name_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yyqq/Documents/liyang/scripts/start_2/start2/configuration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB001099-6D9D-0A4D-983B-2134B71FB95A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BDA9A0B-7175-AE4D-8CE6-2480F45FFD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4880" yWindow="500" windowWidth="46320" windowHeight="26640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
   <si>
     <t>email</t>
   </si>
@@ -80,9 +80,6 @@
   </si>
   <si>
     <t>4536 位置3</t>
-  </si>
-  <si>
-    <t>liyang.tjtj@gmail.com</t>
   </si>
   <si>
     <t>2917 位置4</t>
@@ -617,19 +614,15 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="2"/>
+      <c r="H5" t="s">
         <v>20</v>
       </c>
-      <c r="H5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="H6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I6" t="s">
         <v>18</v>
@@ -637,76 +630,76 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>24</v>
-      </c>
-      <c r="C7" t="s">
-        <v>25</v>
       </c>
       <c r="D7" s="3">
         <v>45699.982743055552</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F7" s="3">
         <v>45658.982743055552</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I7" s="2"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G8" s="2"/>
       <c r="H8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G9" s="2"/>
       <c r="H9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G10" s="2"/>
       <c r="H10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G11" s="2"/>
       <c r="H11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I11" s="2"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
         <v>32</v>
-      </c>
-      <c r="C12" t="s">
-        <v>33</v>
       </c>
       <c r="D12" s="3">
         <v>45658.982743055552</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F12" s="3">
         <v>45658.982743055552</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I12"/>
     </row>
@@ -724,35 +717,35 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" t="s">
         <v>36</v>
-      </c>
-      <c r="C17" t="s">
-        <v>37</v>
       </c>
       <c r="D17" s="3">
         <v>45658.982743055552</v>
       </c>
       <c r="E17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F17" s="3">
         <v>45658.982743055552</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I17" s="2"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="H18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I18" s="2"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update config for zzj7810715@iCloud.com
</commit_message>
<xml_diff>
--- a/configuration/name_list.xlsx
+++ b/configuration/name_list.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4880" yWindow="500" windowWidth="46320" windowHeight="26640" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="list" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="list" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -588,7 +588,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>zzj7810715@iCloud.com</t>
+        </is>
+      </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
           <t>2917 位置4</t>

</xml_diff>

<commit_message>
Revert "update config for liyang.tjtj@gmail.com"
This reverts commit 6d0abd5efcd42fc72b5f1791f60d9841c9f99926.
</commit_message>
<xml_diff>
--- a/configuration/name_list.xlsx
+++ b/configuration/name_list.xlsx
@@ -649,11 +649,7 @@
           <t>1311 位置1</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>liyang.tjtj@gmail.com</t>
-        </is>
-      </c>
+      <c r="I7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="G8" s="2" t="n"/>

</xml_diff>

<commit_message>
update config for y67877687866231y@gmail.com
</commit_message>
<xml_diff>
--- a/configuration/name_list.xlsx
+++ b/configuration/name_list.xlsx
@@ -649,7 +649,11 @@
           <t>1311 位置1</t>
         </is>
       </c>
-      <c r="I7" s="2" t="n"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>y67877687866231y@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="G8" s="2" t="n"/>

</xml_diff>

<commit_message>
update config for 479697929@qq.com
</commit_message>
<xml_diff>
--- a/configuration/name_list.xlsx
+++ b/configuration/name_list.xlsx
@@ -667,7 +667,11 @@
           <t>8374 位置2</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>479697929@qq.com</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="G9" s="2" t="n"/>

</xml_diff>

<commit_message>
update config for leo@alu.scu.edu.cn
</commit_message>
<xml_diff>
--- a/configuration/name_list.xlsx
+++ b/configuration/name_list.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="list" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="list" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -675,7 +675,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="G8" s="4" t="n"/>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>leo@alu.scu.edu.cn</t>
+        </is>
+      </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
           <t>8374 位置2</t>
@@ -694,7 +698,11 @@
           <t>8694 位置3</t>
         </is>
       </c>
-      <c r="I9" s="4" t="n"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>leo@alu.scu.edu.cn</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="G10" s="4" t="n"/>

</xml_diff>

<commit_message>
regenerate update config for ln52601314@qq.com
</commit_message>
<xml_diff>
--- a/configuration/name_list.xlsx
+++ b/configuration/name_list.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4880" yWindow="500" windowWidth="46320" windowHeight="26640" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="list" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="list" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -701,7 +701,11 @@
           <t>1292 位置4</t>
         </is>
       </c>
-      <c r="I10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>ln52601314@qq.com</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="G11" s="2" t="n"/>
@@ -749,7 +753,7 @@
     </row>
     <row r="13">
       <c r="G13" s="2" t="n"/>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="0" t="inlineStr">
         <is>
           <t>6169 位置2</t>
         </is>
@@ -757,7 +761,7 @@
     </row>
     <row r="14">
       <c r="G14" s="2" t="n"/>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="0" t="inlineStr">
         <is>
           <t>6188 位置3</t>
         </is>
@@ -765,7 +769,7 @@
     </row>
     <row r="15">
       <c r="G15" s="2" t="n"/>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="0" t="inlineStr">
         <is>
           <t>1266 位置4</t>
         </is>
@@ -773,7 +777,7 @@
     </row>
     <row r="16">
       <c r="G16" s="2" t="n"/>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="0" t="inlineStr">
         <is>
           <t>6226 位置5</t>
         </is>
@@ -818,21 +822,21 @@
       <c r="I18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="0" t="inlineStr">
         <is>
           <t>1650 位置3</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="0" t="inlineStr">
         <is>
           <t>3295 位置4</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="0" t="inlineStr">
         <is>
           <t>1714 位置5</t>
         </is>

</xml_diff>